<commit_message>
improved logs; added multipliers
</commit_message>
<xml_diff>
--- a/resultado_oficial_oitavas.xlsx
+++ b/resultado_oficial_oitavas.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="34">
   <si>
     <t xml:space="preserve">OITAVAS DE FINAL</t>
   </si>
@@ -57,6 +57,9 @@
   </si>
   <si>
     <t xml:space="preserve">VENCEDOR APOS TEMPO REGULAMENTAR (MARCAR X NA EQUIPE VENCEDORA)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PONTOS (NAO PREENCHER)</t>
   </si>
   <si>
     <t xml:space="preserve">Czechia</t>
@@ -224,7 +227,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -270,7 +273,13 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF999999"/>
-        <bgColor rgb="FF808080"/>
+        <bgColor rgb="FFB2B2B2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFB2B2B2"/>
+        <bgColor rgb="FF999999"/>
       </patternFill>
     </fill>
   </fills>
@@ -343,7 +352,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="38">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -412,6 +421,10 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="true"/>
+    </xf>
     <xf numFmtId="164" fontId="9" fillId="6" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -436,6 +449,10 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="false" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="11" fillId="9" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="9" fillId="2" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -472,19 +489,19 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -552,7 +569,7 @@
       <rgbColor rgb="FF808000"/>
       <rgbColor rgb="FF800080"/>
       <rgbColor rgb="FF008080"/>
-      <rgbColor rgb="FFC0C0C0"/>
+      <rgbColor rgb="FFB2B2B2"/>
       <rgbColor rgb="FF808080"/>
       <rgbColor rgb="FF9999FF"/>
       <rgbColor rgb="FF993366"/>
@@ -722,7 +739,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="42.75"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="23.09"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="24.76"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="54.12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="36.03"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="85.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -883,7 +900,9 @@
         <v>11</v>
       </c>
       <c r="J4" s="16"/>
-      <c r="K4" s="13"/>
+      <c r="K4" s="17" t="s">
+        <v>12</v>
+      </c>
       <c r="L4" s="13"/>
       <c r="M4" s="13"/>
       <c r="N4" s="13"/>
@@ -898,29 +917,29 @@
     </row>
     <row r="5" customFormat="false" ht="24.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="13"/>
-      <c r="B5" s="17" t="n">
+      <c r="B5" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="C5" s="18"/>
-      <c r="D5" s="19" t="s">
-        <v>12</v>
-      </c>
-      <c r="E5" s="19" t="s">
+      <c r="C5" s="19"/>
+      <c r="D5" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="F5" s="20" t="n">
+      <c r="E5" s="20" t="s">
+        <v>14</v>
+      </c>
+      <c r="F5" s="21" t="n">
         <v>2</v>
       </c>
-      <c r="G5" s="20" t="n">
+      <c r="G5" s="21" t="n">
         <v>1</v>
       </c>
-      <c r="H5" s="21" t="str">
+      <c r="H5" s="22" t="str">
         <f aca="false">IF(OR(ISBLANK(F5) , ISBLANK(G5)),"?",IF(F5&gt;G5,D5,IF(G5&gt;F5,E5,IF(AND(ISBLANK(J5), OR(I5 = "X",I5 = "x")),D5,IF(AND(ISBLANK(I5), OR(J5 = "X",J5 = "x")),E5,"?")))))</f>
         <v>Czechia</v>
       </c>
-      <c r="I5" s="22"/>
-      <c r="J5" s="22"/>
-      <c r="K5" s="13"/>
+      <c r="I5" s="23"/>
+      <c r="J5" s="23"/>
+      <c r="K5" s="24"/>
       <c r="L5" s="13"/>
       <c r="M5" s="13"/>
       <c r="N5" s="13"/>
@@ -935,32 +954,32 @@
     </row>
     <row r="6" customFormat="false" ht="24.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="13"/>
-      <c r="B6" s="17" t="n">
+      <c r="B6" s="18" t="n">
         <f aca="false">+B5+1</f>
         <v>2</v>
       </c>
-      <c r="C6" s="18"/>
-      <c r="D6" s="19" t="s">
+      <c r="C6" s="19"/>
+      <c r="D6" s="20" t="s">
+        <v>15</v>
+      </c>
+      <c r="E6" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="E6" s="19" t="s">
-        <v>13</v>
-      </c>
-      <c r="F6" s="20" t="n">
+      <c r="F6" s="21" t="n">
         <v>3</v>
       </c>
-      <c r="G6" s="20" t="n">
+      <c r="G6" s="21" t="n">
         <v>3</v>
       </c>
-      <c r="H6" s="21" t="str">
+      <c r="H6" s="22" t="str">
         <f aca="false">IF(OR(ISBLANK(F6) , ISBLANK(G6)),"?",IF(F6&gt;G6,D6,IF(G6&gt;F6,E6,IF(AND(ISBLANK(J6), OR(I6 = "X",I6 = "x")),D6,IF(AND(ISBLANK(I6), OR(J6 = "X",J6 = "x")),E6,"?")))))</f>
         <v>South Africa</v>
       </c>
-      <c r="I6" s="22"/>
-      <c r="J6" s="22" t="s">
-        <v>15</v>
-      </c>
-      <c r="K6" s="13"/>
+      <c r="I6" s="23"/>
+      <c r="J6" s="23" t="s">
+        <v>16</v>
+      </c>
+      <c r="K6" s="24"/>
       <c r="L6" s="13"/>
       <c r="M6" s="13"/>
       <c r="N6" s="13"/>
@@ -975,30 +994,30 @@
     </row>
     <row r="7" customFormat="false" ht="24.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="13"/>
-      <c r="B7" s="17" t="n">
+      <c r="B7" s="18" t="n">
         <f aca="false">+B6+1</f>
         <v>3</v>
       </c>
-      <c r="C7" s="18"/>
-      <c r="D7" s="19" t="s">
-        <v>16</v>
-      </c>
-      <c r="E7" s="19" t="s">
-        <v>12</v>
-      </c>
-      <c r="F7" s="20" t="n">
+      <c r="C7" s="19"/>
+      <c r="D7" s="20" t="s">
+        <v>17</v>
+      </c>
+      <c r="E7" s="20" t="s">
+        <v>13</v>
+      </c>
+      <c r="F7" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="G7" s="20" t="n">
+      <c r="G7" s="21" t="n">
         <v>5</v>
       </c>
-      <c r="H7" s="21" t="str">
+      <c r="H7" s="22" t="str">
         <f aca="false">IF(OR(ISBLANK(F7) , ISBLANK(G7)),"?",IF(F7&gt;G7,D7,IF(G7&gt;F7,E7,IF(AND(ISBLANK(J7), OR(I7 = "X",I7 = "x")),D7,IF(AND(ISBLANK(I7), OR(J7 = "X",J7 = "x")),E7,"?")))))</f>
         <v>Czechia</v>
       </c>
-      <c r="I7" s="22"/>
-      <c r="J7" s="22"/>
-      <c r="K7" s="13"/>
+      <c r="I7" s="23"/>
+      <c r="J7" s="23"/>
+      <c r="K7" s="24"/>
       <c r="L7" s="13"/>
       <c r="M7" s="13"/>
       <c r="N7" s="13"/>
@@ -1013,26 +1032,26 @@
     </row>
     <row r="8" customFormat="false" ht="24.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="13"/>
-      <c r="B8" s="17" t="n">
+      <c r="B8" s="18" t="n">
         <f aca="false">+B7+1</f>
         <v>4</v>
       </c>
-      <c r="C8" s="18"/>
-      <c r="D8" s="19" t="s">
-        <v>14</v>
-      </c>
-      <c r="E8" s="19" t="s">
-        <v>16</v>
-      </c>
-      <c r="F8" s="20"/>
-      <c r="G8" s="20"/>
-      <c r="H8" s="21" t="str">
+      <c r="C8" s="19"/>
+      <c r="D8" s="20" t="s">
+        <v>15</v>
+      </c>
+      <c r="E8" s="20" t="s">
+        <v>17</v>
+      </c>
+      <c r="F8" s="21"/>
+      <c r="G8" s="21"/>
+      <c r="H8" s="22" t="str">
         <f aca="false">IF(OR(ISBLANK(F8) , ISBLANK(G8)),"?",IF(F8&gt;G8,D8,IF(G8&gt;F8,E8,IF(AND(ISBLANK(J8), OR(I8 = "X",I8 = "x")),D8,IF(AND(ISBLANK(I8), OR(J8 = "X",J8 = "x")),E8,"?")))))</f>
         <v>?</v>
       </c>
-      <c r="I8" s="22"/>
-      <c r="J8" s="22"/>
-      <c r="K8" s="13"/>
+      <c r="I8" s="23"/>
+      <c r="J8" s="23"/>
+      <c r="K8" s="24"/>
       <c r="L8" s="13"/>
       <c r="M8" s="13"/>
       <c r="N8" s="13"/>
@@ -1047,26 +1066,26 @@
     </row>
     <row r="9" customFormat="false" ht="24.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="13"/>
-      <c r="B9" s="17" t="n">
+      <c r="B9" s="18" t="n">
         <f aca="false">+B8+1</f>
         <v>5</v>
       </c>
-      <c r="C9" s="18"/>
-      <c r="D9" s="19" t="s">
-        <v>12</v>
-      </c>
-      <c r="E9" s="19" t="s">
-        <v>14</v>
-      </c>
-      <c r="F9" s="20"/>
-      <c r="G9" s="20"/>
-      <c r="H9" s="21" t="str">
+      <c r="C9" s="19"/>
+      <c r="D9" s="20" t="s">
+        <v>13</v>
+      </c>
+      <c r="E9" s="20" t="s">
+        <v>15</v>
+      </c>
+      <c r="F9" s="21"/>
+      <c r="G9" s="21"/>
+      <c r="H9" s="22" t="str">
         <f aca="false">IF(OR(ISBLANK(F9) , ISBLANK(G9)),"?",IF(F9&gt;G9,D9,IF(G9&gt;F9,E9,IF(AND(ISBLANK(J9), OR(I9 = "X",I9 = "x")),D9,IF(AND(ISBLANK(I9), OR(J9 = "X",J9 = "x")),E9,"?")))))</f>
         <v>?</v>
       </c>
-      <c r="I9" s="22"/>
-      <c r="J9" s="22"/>
-      <c r="K9" s="13"/>
+      <c r="I9" s="23"/>
+      <c r="J9" s="23"/>
+      <c r="K9" s="24"/>
       <c r="L9" s="13"/>
       <c r="M9" s="13"/>
       <c r="N9" s="13"/>
@@ -1081,32 +1100,32 @@
     </row>
     <row r="10" customFormat="false" ht="24.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="13"/>
-      <c r="B10" s="17" t="n">
+      <c r="B10" s="18" t="n">
         <f aca="false">+B9+1</f>
         <v>6</v>
       </c>
-      <c r="C10" s="18"/>
-      <c r="D10" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="E10" s="19" t="s">
+      <c r="C10" s="19"/>
+      <c r="D10" s="20" t="s">
         <v>18</v>
       </c>
-      <c r="F10" s="20" t="n">
+      <c r="E10" s="20" t="s">
+        <v>19</v>
+      </c>
+      <c r="F10" s="21" t="n">
         <v>2</v>
       </c>
-      <c r="G10" s="20" t="n">
+      <c r="G10" s="21" t="n">
         <v>2</v>
       </c>
-      <c r="H10" s="21" t="str">
+      <c r="H10" s="22" t="str">
         <f aca="false">IF(OR(ISBLANK(F10) , ISBLANK(G10)),"?",IF(F10&gt;G10,D10,IF(G10&gt;F10,E10,IF(AND(ISBLANK(J10), OR(I10 = "X",I10 = "x")),D10,IF(AND(ISBLANK(I10), OR(J10 = "X",J10 = "x")),E10,"?")))))</f>
         <v>TIME A</v>
       </c>
-      <c r="I10" s="22" t="s">
-        <v>19</v>
-      </c>
-      <c r="J10" s="22"/>
-      <c r="K10" s="13"/>
+      <c r="I10" s="23" t="s">
+        <v>20</v>
+      </c>
+      <c r="J10" s="23"/>
+      <c r="K10" s="24"/>
       <c r="L10" s="13"/>
       <c r="M10" s="13"/>
       <c r="N10" s="13"/>
@@ -1121,26 +1140,26 @@
     </row>
     <row r="11" customFormat="false" ht="24.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="13"/>
-      <c r="B11" s="17" t="n">
+      <c r="B11" s="18" t="n">
         <f aca="false">+B10+1</f>
         <v>7</v>
       </c>
-      <c r="C11" s="18"/>
-      <c r="D11" s="19" t="s">
-        <v>20</v>
-      </c>
-      <c r="E11" s="19" t="s">
+      <c r="C11" s="19"/>
+      <c r="D11" s="20" t="s">
         <v>21</v>
       </c>
-      <c r="F11" s="20"/>
-      <c r="G11" s="20"/>
-      <c r="H11" s="21" t="str">
+      <c r="E11" s="20" t="s">
+        <v>22</v>
+      </c>
+      <c r="F11" s="21"/>
+      <c r="G11" s="21"/>
+      <c r="H11" s="22" t="str">
         <f aca="false">IF(OR(ISBLANK(F11) , ISBLANK(G11)),"?",IF(F11&gt;G11,D11,IF(G11&gt;F11,E11,IF(AND(ISBLANK(J11), OR(I11 = "X",I11 = "x")),D11,IF(AND(ISBLANK(I11), OR(J11 = "X",J11 = "x")),E11,"?")))))</f>
         <v>?</v>
       </c>
-      <c r="I11" s="22"/>
-      <c r="J11" s="22"/>
-      <c r="K11" s="13"/>
+      <c r="I11" s="23"/>
+      <c r="J11" s="23"/>
+      <c r="K11" s="24"/>
       <c r="L11" s="13"/>
       <c r="M11" s="13"/>
       <c r="N11" s="13"/>
@@ -1155,26 +1174,26 @@
     </row>
     <row r="12" customFormat="false" ht="24.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="13"/>
-      <c r="B12" s="17" t="n">
+      <c r="B12" s="18" t="n">
         <f aca="false">+B11+1</f>
         <v>8</v>
       </c>
-      <c r="C12" s="18"/>
-      <c r="D12" s="19" t="s">
-        <v>22</v>
-      </c>
-      <c r="E12" s="19" t="s">
+      <c r="C12" s="19"/>
+      <c r="D12" s="20" t="s">
         <v>23</v>
       </c>
-      <c r="F12" s="20"/>
-      <c r="G12" s="20"/>
-      <c r="H12" s="21" t="str">
+      <c r="E12" s="20" t="s">
+        <v>24</v>
+      </c>
+      <c r="F12" s="21"/>
+      <c r="G12" s="21"/>
+      <c r="H12" s="22" t="str">
         <f aca="false">IF(OR(ISBLANK(F12) , ISBLANK(G12)),"?",IF(F12&gt;G12,D12,IF(G12&gt;F12,E12,IF(AND(ISBLANK(J12), OR(I12 = "X",I12 = "x")),D12,IF(AND(ISBLANK(I12), OR(J12 = "X",J12 = "x")),E12,"?")))))</f>
         <v>?</v>
       </c>
-      <c r="I12" s="22"/>
-      <c r="J12" s="22"/>
-      <c r="K12" s="13"/>
+      <c r="I12" s="23"/>
+      <c r="J12" s="23"/>
+      <c r="K12" s="24"/>
       <c r="L12" s="13"/>
       <c r="M12" s="13"/>
       <c r="N12" s="13"/>
@@ -1189,15 +1208,15 @@
     </row>
     <row r="13" customFormat="false" ht="24.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="13"/>
-      <c r="B13" s="23"/>
-      <c r="C13" s="24"/>
-      <c r="D13" s="25"/>
-      <c r="E13" s="25"/>
-      <c r="F13" s="26"/>
-      <c r="G13" s="26"/>
-      <c r="H13" s="27"/>
-      <c r="I13" s="28"/>
-      <c r="J13" s="28"/>
+      <c r="B13" s="25"/>
+      <c r="C13" s="26"/>
+      <c r="D13" s="27"/>
+      <c r="E13" s="27"/>
+      <c r="F13" s="28"/>
+      <c r="G13" s="28"/>
+      <c r="H13" s="29"/>
+      <c r="I13" s="30"/>
+      <c r="J13" s="30"/>
       <c r="K13" s="13"/>
       <c r="L13" s="13"/>
       <c r="M13" s="13"/>
@@ -1213,15 +1232,15 @@
     </row>
     <row r="14" customFormat="false" ht="24.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="13"/>
-      <c r="B14" s="23"/>
-      <c r="C14" s="24"/>
-      <c r="D14" s="25"/>
-      <c r="E14" s="25"/>
-      <c r="F14" s="26"/>
-      <c r="G14" s="26"/>
-      <c r="H14" s="27"/>
-      <c r="I14" s="28"/>
-      <c r="J14" s="28"/>
+      <c r="B14" s="25"/>
+      <c r="C14" s="26"/>
+      <c r="D14" s="27"/>
+      <c r="E14" s="27"/>
+      <c r="F14" s="28"/>
+      <c r="G14" s="28"/>
+      <c r="H14" s="29"/>
+      <c r="I14" s="30"/>
+      <c r="J14" s="30"/>
       <c r="K14" s="13"/>
       <c r="L14" s="13"/>
       <c r="M14" s="13"/>
@@ -1237,15 +1256,15 @@
     </row>
     <row r="15" customFormat="false" ht="24.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="13"/>
-      <c r="B15" s="23"/>
-      <c r="C15" s="24"/>
-      <c r="D15" s="25"/>
-      <c r="E15" s="25"/>
-      <c r="F15" s="26"/>
-      <c r="G15" s="26"/>
-      <c r="H15" s="27"/>
-      <c r="I15" s="28"/>
-      <c r="J15" s="28"/>
+      <c r="B15" s="25"/>
+      <c r="C15" s="26"/>
+      <c r="D15" s="27"/>
+      <c r="E15" s="27"/>
+      <c r="F15" s="28"/>
+      <c r="G15" s="28"/>
+      <c r="H15" s="29"/>
+      <c r="I15" s="30"/>
+      <c r="J15" s="30"/>
       <c r="K15" s="13"/>
       <c r="L15" s="13"/>
       <c r="M15" s="13"/>
@@ -1261,15 +1280,15 @@
     </row>
     <row r="16" customFormat="false" ht="24.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="13"/>
-      <c r="B16" s="23"/>
-      <c r="C16" s="24"/>
-      <c r="D16" s="25"/>
-      <c r="E16" s="25"/>
-      <c r="F16" s="26"/>
-      <c r="G16" s="26"/>
-      <c r="H16" s="27"/>
-      <c r="I16" s="28"/>
-      <c r="J16" s="28"/>
+      <c r="B16" s="25"/>
+      <c r="C16" s="26"/>
+      <c r="D16" s="27"/>
+      <c r="E16" s="27"/>
+      <c r="F16" s="28"/>
+      <c r="G16" s="28"/>
+      <c r="H16" s="29"/>
+      <c r="I16" s="30"/>
+      <c r="J16" s="30"/>
       <c r="K16" s="13"/>
       <c r="L16" s="13"/>
       <c r="M16" s="13"/>
@@ -1285,15 +1304,15 @@
     </row>
     <row r="17" customFormat="false" ht="24.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="13"/>
-      <c r="B17" s="23"/>
-      <c r="C17" s="24"/>
-      <c r="D17" s="25"/>
-      <c r="E17" s="25"/>
-      <c r="F17" s="26"/>
-      <c r="G17" s="26"/>
-      <c r="H17" s="27"/>
-      <c r="I17" s="28"/>
-      <c r="J17" s="28"/>
+      <c r="B17" s="25"/>
+      <c r="C17" s="26"/>
+      <c r="D17" s="27"/>
+      <c r="E17" s="27"/>
+      <c r="F17" s="28"/>
+      <c r="G17" s="28"/>
+      <c r="H17" s="29"/>
+      <c r="I17" s="30"/>
+      <c r="J17" s="30"/>
       <c r="K17" s="13"/>
       <c r="L17" s="13"/>
       <c r="M17" s="13"/>
@@ -1309,15 +1328,15 @@
     </row>
     <row r="18" customFormat="false" ht="24.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="13"/>
-      <c r="B18" s="23"/>
-      <c r="C18" s="24"/>
-      <c r="D18" s="25"/>
-      <c r="E18" s="25"/>
-      <c r="F18" s="26"/>
-      <c r="G18" s="26"/>
-      <c r="H18" s="27"/>
-      <c r="I18" s="28"/>
-      <c r="J18" s="28"/>
+      <c r="B18" s="25"/>
+      <c r="C18" s="26"/>
+      <c r="D18" s="27"/>
+      <c r="E18" s="27"/>
+      <c r="F18" s="28"/>
+      <c r="G18" s="28"/>
+      <c r="H18" s="29"/>
+      <c r="I18" s="30"/>
+      <c r="J18" s="30"/>
       <c r="K18" s="13"/>
       <c r="L18" s="13"/>
       <c r="M18" s="13"/>
@@ -1333,15 +1352,15 @@
     </row>
     <row r="19" customFormat="false" ht="24.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="13"/>
-      <c r="B19" s="23"/>
-      <c r="C19" s="24"/>
-      <c r="D19" s="25"/>
-      <c r="E19" s="25"/>
-      <c r="F19" s="26"/>
-      <c r="G19" s="26"/>
-      <c r="H19" s="27"/>
-      <c r="I19" s="28"/>
-      <c r="J19" s="28"/>
+      <c r="B19" s="25"/>
+      <c r="C19" s="26"/>
+      <c r="D19" s="27"/>
+      <c r="E19" s="27"/>
+      <c r="F19" s="28"/>
+      <c r="G19" s="28"/>
+      <c r="H19" s="29"/>
+      <c r="I19" s="30"/>
+      <c r="J19" s="30"/>
       <c r="K19" s="13"/>
       <c r="L19" s="13"/>
       <c r="M19" s="13"/>
@@ -1357,15 +1376,15 @@
     </row>
     <row r="20" customFormat="false" ht="24.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="13"/>
-      <c r="B20" s="23"/>
-      <c r="C20" s="24"/>
-      <c r="D20" s="25"/>
-      <c r="E20" s="25"/>
-      <c r="F20" s="26"/>
-      <c r="G20" s="26"/>
-      <c r="H20" s="27"/>
-      <c r="I20" s="28"/>
-      <c r="J20" s="28"/>
+      <c r="B20" s="25"/>
+      <c r="C20" s="26"/>
+      <c r="D20" s="27"/>
+      <c r="E20" s="27"/>
+      <c r="F20" s="28"/>
+      <c r="G20" s="28"/>
+      <c r="H20" s="29"/>
+      <c r="I20" s="30"/>
+      <c r="J20" s="30"/>
       <c r="K20" s="13"/>
       <c r="L20" s="13"/>
       <c r="M20" s="13"/>
@@ -1381,15 +1400,15 @@
     </row>
     <row r="21" customFormat="false" ht="24.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="13"/>
-      <c r="B21" s="23"/>
-      <c r="C21" s="24"/>
-      <c r="D21" s="25"/>
-      <c r="E21" s="25"/>
-      <c r="F21" s="26"/>
-      <c r="G21" s="26"/>
-      <c r="H21" s="27"/>
-      <c r="I21" s="28"/>
-      <c r="J21" s="28"/>
+      <c r="B21" s="25"/>
+      <c r="C21" s="26"/>
+      <c r="D21" s="27"/>
+      <c r="E21" s="27"/>
+      <c r="F21" s="28"/>
+      <c r="G21" s="28"/>
+      <c r="H21" s="29"/>
+      <c r="I21" s="30"/>
+      <c r="J21" s="30"/>
       <c r="K21" s="13"/>
       <c r="L21" s="13"/>
       <c r="M21" s="13"/>
@@ -1405,15 +1424,15 @@
     </row>
     <row r="22" customFormat="false" ht="24.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="13"/>
-      <c r="B22" s="23"/>
-      <c r="C22" s="24"/>
-      <c r="D22" s="25"/>
-      <c r="E22" s="25"/>
-      <c r="F22" s="26"/>
-      <c r="G22" s="26"/>
-      <c r="H22" s="27"/>
-      <c r="I22" s="28"/>
-      <c r="J22" s="28"/>
+      <c r="B22" s="25"/>
+      <c r="C22" s="26"/>
+      <c r="D22" s="27"/>
+      <c r="E22" s="27"/>
+      <c r="F22" s="28"/>
+      <c r="G22" s="28"/>
+      <c r="H22" s="29"/>
+      <c r="I22" s="30"/>
+      <c r="J22" s="30"/>
       <c r="K22" s="13"/>
       <c r="L22" s="13"/>
       <c r="M22" s="13"/>
@@ -1429,15 +1448,15 @@
     </row>
     <row r="23" customFormat="false" ht="24.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="13"/>
-      <c r="B23" s="23"/>
-      <c r="C23" s="24"/>
-      <c r="D23" s="25"/>
-      <c r="E23" s="25"/>
-      <c r="F23" s="26"/>
-      <c r="G23" s="26"/>
-      <c r="H23" s="27"/>
-      <c r="I23" s="28"/>
-      <c r="J23" s="28"/>
+      <c r="B23" s="25"/>
+      <c r="C23" s="26"/>
+      <c r="D23" s="27"/>
+      <c r="E23" s="27"/>
+      <c r="F23" s="28"/>
+      <c r="G23" s="28"/>
+      <c r="H23" s="29"/>
+      <c r="I23" s="30"/>
+      <c r="J23" s="30"/>
       <c r="K23" s="13"/>
       <c r="L23" s="13"/>
       <c r="M23" s="13"/>
@@ -1453,15 +1472,15 @@
     </row>
     <row r="24" customFormat="false" ht="24.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="13"/>
-      <c r="B24" s="23"/>
-      <c r="C24" s="24"/>
-      <c r="D24" s="25"/>
-      <c r="E24" s="25"/>
-      <c r="F24" s="26"/>
-      <c r="G24" s="26"/>
-      <c r="H24" s="27"/>
-      <c r="I24" s="28"/>
-      <c r="J24" s="28"/>
+      <c r="B24" s="25"/>
+      <c r="C24" s="26"/>
+      <c r="D24" s="27"/>
+      <c r="E24" s="27"/>
+      <c r="F24" s="28"/>
+      <c r="G24" s="28"/>
+      <c r="H24" s="29"/>
+      <c r="I24" s="30"/>
+      <c r="J24" s="30"/>
       <c r="K24" s="13"/>
       <c r="L24" s="13"/>
       <c r="M24" s="13"/>
@@ -1477,15 +1496,15 @@
     </row>
     <row r="25" customFormat="false" ht="24.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="13"/>
-      <c r="B25" s="23"/>
-      <c r="C25" s="24"/>
-      <c r="D25" s="25"/>
-      <c r="E25" s="25"/>
-      <c r="F25" s="26"/>
-      <c r="G25" s="26"/>
-      <c r="H25" s="27"/>
-      <c r="I25" s="28"/>
-      <c r="J25" s="28"/>
+      <c r="B25" s="25"/>
+      <c r="C25" s="26"/>
+      <c r="D25" s="27"/>
+      <c r="E25" s="27"/>
+      <c r="F25" s="28"/>
+      <c r="G25" s="28"/>
+      <c r="H25" s="29"/>
+      <c r="I25" s="30"/>
+      <c r="J25" s="30"/>
       <c r="K25" s="13"/>
       <c r="L25" s="13"/>
       <c r="M25" s="13"/>
@@ -1501,15 +1520,15 @@
     </row>
     <row r="26" customFormat="false" ht="24.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="13"/>
-      <c r="B26" s="23"/>
-      <c r="C26" s="24"/>
-      <c r="D26" s="25"/>
-      <c r="E26" s="25"/>
-      <c r="F26" s="26"/>
-      <c r="G26" s="26"/>
-      <c r="H26" s="27"/>
-      <c r="I26" s="28"/>
-      <c r="J26" s="28"/>
+      <c r="B26" s="25"/>
+      <c r="C26" s="26"/>
+      <c r="D26" s="27"/>
+      <c r="E26" s="27"/>
+      <c r="F26" s="28"/>
+      <c r="G26" s="28"/>
+      <c r="H26" s="29"/>
+      <c r="I26" s="30"/>
+      <c r="J26" s="30"/>
       <c r="K26" s="13"/>
       <c r="L26" s="13"/>
       <c r="M26" s="13"/>
@@ -1525,15 +1544,15 @@
     </row>
     <row r="27" customFormat="false" ht="24.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="13"/>
-      <c r="B27" s="23"/>
-      <c r="C27" s="24"/>
-      <c r="D27" s="25"/>
-      <c r="E27" s="25"/>
-      <c r="F27" s="26"/>
-      <c r="G27" s="26"/>
-      <c r="H27" s="27"/>
-      <c r="I27" s="28"/>
-      <c r="J27" s="28"/>
+      <c r="B27" s="25"/>
+      <c r="C27" s="26"/>
+      <c r="D27" s="27"/>
+      <c r="E27" s="27"/>
+      <c r="F27" s="28"/>
+      <c r="G27" s="28"/>
+      <c r="H27" s="29"/>
+      <c r="I27" s="30"/>
+      <c r="J27" s="30"/>
       <c r="K27" s="13"/>
       <c r="L27" s="13"/>
       <c r="M27" s="13"/>
@@ -1549,15 +1568,15 @@
     </row>
     <row r="28" customFormat="false" ht="24.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="13"/>
-      <c r="B28" s="23"/>
-      <c r="C28" s="24"/>
-      <c r="D28" s="25"/>
-      <c r="E28" s="25"/>
-      <c r="F28" s="26"/>
-      <c r="G28" s="26"/>
-      <c r="H28" s="27"/>
-      <c r="I28" s="28"/>
-      <c r="J28" s="28"/>
+      <c r="B28" s="25"/>
+      <c r="C28" s="26"/>
+      <c r="D28" s="27"/>
+      <c r="E28" s="27"/>
+      <c r="F28" s="28"/>
+      <c r="G28" s="28"/>
+      <c r="H28" s="29"/>
+      <c r="I28" s="30"/>
+      <c r="J28" s="30"/>
       <c r="K28" s="13"/>
       <c r="L28" s="13"/>
       <c r="M28" s="13"/>
@@ -1573,15 +1592,15 @@
     </row>
     <row r="29" customFormat="false" ht="24.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="13"/>
-      <c r="B29" s="23"/>
-      <c r="C29" s="24"/>
-      <c r="D29" s="25"/>
-      <c r="E29" s="25"/>
-      <c r="F29" s="26"/>
-      <c r="G29" s="26"/>
-      <c r="H29" s="27"/>
-      <c r="I29" s="28"/>
-      <c r="J29" s="28"/>
+      <c r="B29" s="25"/>
+      <c r="C29" s="26"/>
+      <c r="D29" s="27"/>
+      <c r="E29" s="27"/>
+      <c r="F29" s="28"/>
+      <c r="G29" s="28"/>
+      <c r="H29" s="29"/>
+      <c r="I29" s="30"/>
+      <c r="J29" s="30"/>
       <c r="K29" s="13"/>
       <c r="L29" s="13"/>
       <c r="M29" s="13"/>
@@ -1597,15 +1616,15 @@
     </row>
     <row r="30" customFormat="false" ht="24.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="13"/>
-      <c r="B30" s="23"/>
-      <c r="C30" s="24"/>
-      <c r="D30" s="25"/>
-      <c r="E30" s="25"/>
-      <c r="F30" s="26"/>
-      <c r="G30" s="26"/>
-      <c r="H30" s="27"/>
-      <c r="I30" s="28"/>
-      <c r="J30" s="28"/>
+      <c r="B30" s="25"/>
+      <c r="C30" s="26"/>
+      <c r="D30" s="27"/>
+      <c r="E30" s="27"/>
+      <c r="F30" s="28"/>
+      <c r="G30" s="28"/>
+      <c r="H30" s="29"/>
+      <c r="I30" s="30"/>
+      <c r="J30" s="30"/>
       <c r="K30" s="13"/>
       <c r="L30" s="13"/>
       <c r="M30" s="13"/>
@@ -1621,15 +1640,15 @@
     </row>
     <row r="31" customFormat="false" ht="24.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="13"/>
-      <c r="B31" s="23"/>
-      <c r="C31" s="24"/>
-      <c r="D31" s="25"/>
-      <c r="E31" s="25"/>
-      <c r="F31" s="26"/>
-      <c r="G31" s="26"/>
-      <c r="H31" s="27"/>
-      <c r="I31" s="28"/>
-      <c r="J31" s="28"/>
+      <c r="B31" s="25"/>
+      <c r="C31" s="26"/>
+      <c r="D31" s="27"/>
+      <c r="E31" s="27"/>
+      <c r="F31" s="28"/>
+      <c r="G31" s="28"/>
+      <c r="H31" s="29"/>
+      <c r="I31" s="30"/>
+      <c r="J31" s="30"/>
       <c r="K31" s="13"/>
       <c r="L31" s="13"/>
       <c r="M31" s="13"/>
@@ -1645,15 +1664,15 @@
     </row>
     <row r="32" customFormat="false" ht="24.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="13"/>
-      <c r="B32" s="23"/>
-      <c r="C32" s="24"/>
-      <c r="D32" s="25"/>
-      <c r="E32" s="25"/>
-      <c r="F32" s="26"/>
-      <c r="G32" s="26"/>
-      <c r="H32" s="27"/>
-      <c r="I32" s="28"/>
-      <c r="J32" s="28"/>
+      <c r="B32" s="25"/>
+      <c r="C32" s="26"/>
+      <c r="D32" s="27"/>
+      <c r="E32" s="27"/>
+      <c r="F32" s="28"/>
+      <c r="G32" s="28"/>
+      <c r="H32" s="29"/>
+      <c r="I32" s="30"/>
+      <c r="J32" s="30"/>
       <c r="K32" s="13"/>
       <c r="L32" s="13"/>
       <c r="M32" s="13"/>
@@ -1669,15 +1688,15 @@
     </row>
     <row r="33" customFormat="false" ht="24.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="13"/>
-      <c r="B33" s="23"/>
-      <c r="C33" s="24"/>
-      <c r="D33" s="25"/>
-      <c r="E33" s="25"/>
-      <c r="F33" s="26"/>
-      <c r="G33" s="26"/>
-      <c r="H33" s="27"/>
-      <c r="I33" s="28"/>
-      <c r="J33" s="28"/>
+      <c r="B33" s="25"/>
+      <c r="C33" s="26"/>
+      <c r="D33" s="27"/>
+      <c r="E33" s="27"/>
+      <c r="F33" s="28"/>
+      <c r="G33" s="28"/>
+      <c r="H33" s="29"/>
+      <c r="I33" s="30"/>
+      <c r="J33" s="30"/>
       <c r="K33" s="13"/>
       <c r="L33" s="13"/>
       <c r="M33" s="13"/>
@@ -1693,15 +1712,15 @@
     </row>
     <row r="34" customFormat="false" ht="24.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="13"/>
-      <c r="B34" s="23"/>
-      <c r="C34" s="24"/>
-      <c r="D34" s="25"/>
-      <c r="E34" s="25"/>
-      <c r="F34" s="26"/>
-      <c r="G34" s="26"/>
-      <c r="H34" s="27"/>
-      <c r="I34" s="28"/>
-      <c r="J34" s="28"/>
+      <c r="B34" s="25"/>
+      <c r="C34" s="26"/>
+      <c r="D34" s="27"/>
+      <c r="E34" s="27"/>
+      <c r="F34" s="28"/>
+      <c r="G34" s="28"/>
+      <c r="H34" s="29"/>
+      <c r="I34" s="30"/>
+      <c r="J34" s="30"/>
       <c r="K34" s="13"/>
       <c r="L34" s="13"/>
       <c r="M34" s="13"/>
@@ -1717,15 +1736,15 @@
     </row>
     <row r="35" customFormat="false" ht="24.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="13"/>
-      <c r="B35" s="23"/>
-      <c r="C35" s="24"/>
-      <c r="D35" s="25"/>
-      <c r="E35" s="25"/>
-      <c r="F35" s="26"/>
-      <c r="G35" s="26"/>
-      <c r="H35" s="27"/>
-      <c r="I35" s="28"/>
-      <c r="J35" s="28"/>
+      <c r="B35" s="25"/>
+      <c r="C35" s="26"/>
+      <c r="D35" s="27"/>
+      <c r="E35" s="27"/>
+      <c r="F35" s="28"/>
+      <c r="G35" s="28"/>
+      <c r="H35" s="29"/>
+      <c r="I35" s="30"/>
+      <c r="J35" s="30"/>
       <c r="K35" s="13"/>
       <c r="L35" s="13"/>
       <c r="M35" s="13"/>
@@ -1741,15 +1760,15 @@
     </row>
     <row r="36" customFormat="false" ht="24.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="13"/>
-      <c r="B36" s="23"/>
-      <c r="C36" s="24"/>
-      <c r="D36" s="25"/>
-      <c r="E36" s="25"/>
-      <c r="F36" s="26"/>
-      <c r="G36" s="26"/>
-      <c r="H36" s="27"/>
-      <c r="I36" s="28"/>
-      <c r="J36" s="28"/>
+      <c r="B36" s="25"/>
+      <c r="C36" s="26"/>
+      <c r="D36" s="27"/>
+      <c r="E36" s="27"/>
+      <c r="F36" s="28"/>
+      <c r="G36" s="28"/>
+      <c r="H36" s="29"/>
+      <c r="I36" s="30"/>
+      <c r="J36" s="30"/>
       <c r="K36" s="13"/>
       <c r="L36" s="13"/>
       <c r="M36" s="13"/>
@@ -1765,13 +1784,13 @@
     </row>
     <row r="37" customFormat="false" ht="24.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="13"/>
-      <c r="B37" s="23"/>
-      <c r="C37" s="24"/>
-      <c r="D37" s="25"/>
-      <c r="E37" s="25"/>
-      <c r="F37" s="29"/>
-      <c r="G37" s="29"/>
-      <c r="H37" s="27"/>
+      <c r="B37" s="25"/>
+      <c r="C37" s="26"/>
+      <c r="D37" s="27"/>
+      <c r="E37" s="27"/>
+      <c r="F37" s="31"/>
+      <c r="G37" s="31"/>
+      <c r="H37" s="29"/>
       <c r="I37" s="13"/>
       <c r="J37" s="13"/>
       <c r="K37" s="13"/>
@@ -1789,13 +1808,13 @@
     </row>
     <row r="38" customFormat="false" ht="24.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="13"/>
-      <c r="B38" s="23"/>
-      <c r="C38" s="24"/>
-      <c r="D38" s="25"/>
-      <c r="E38" s="25"/>
-      <c r="F38" s="29"/>
-      <c r="G38" s="29"/>
-      <c r="H38" s="27"/>
+      <c r="B38" s="25"/>
+      <c r="C38" s="26"/>
+      <c r="D38" s="27"/>
+      <c r="E38" s="27"/>
+      <c r="F38" s="31"/>
+      <c r="G38" s="31"/>
+      <c r="H38" s="29"/>
       <c r="I38" s="13"/>
       <c r="J38" s="13"/>
       <c r="K38" s="13"/>
@@ -1813,13 +1832,13 @@
     </row>
     <row r="39" customFormat="false" ht="24.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="13"/>
-      <c r="B39" s="23"/>
-      <c r="C39" s="24"/>
-      <c r="D39" s="25"/>
-      <c r="E39" s="25"/>
-      <c r="F39" s="29"/>
-      <c r="G39" s="29"/>
-      <c r="H39" s="27"/>
+      <c r="B39" s="25"/>
+      <c r="C39" s="26"/>
+      <c r="D39" s="27"/>
+      <c r="E39" s="27"/>
+      <c r="F39" s="31"/>
+      <c r="G39" s="31"/>
+      <c r="H39" s="29"/>
       <c r="I39" s="13"/>
       <c r="J39" s="13"/>
       <c r="K39" s="13"/>
@@ -1837,13 +1856,13 @@
     </row>
     <row r="40" customFormat="false" ht="24.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="13"/>
-      <c r="B40" s="23"/>
-      <c r="C40" s="24"/>
-      <c r="D40" s="25"/>
-      <c r="E40" s="25"/>
-      <c r="F40" s="29"/>
-      <c r="G40" s="29"/>
-      <c r="H40" s="27"/>
+      <c r="B40" s="25"/>
+      <c r="C40" s="26"/>
+      <c r="D40" s="27"/>
+      <c r="E40" s="27"/>
+      <c r="F40" s="31"/>
+      <c r="G40" s="31"/>
+      <c r="H40" s="29"/>
       <c r="I40" s="13"/>
       <c r="J40" s="13"/>
       <c r="K40" s="13"/>
@@ -1861,13 +1880,13 @@
     </row>
     <row r="41" customFormat="false" ht="24.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="13"/>
-      <c r="B41" s="23"/>
-      <c r="C41" s="24"/>
-      <c r="D41" s="25"/>
-      <c r="E41" s="25"/>
-      <c r="F41" s="29"/>
-      <c r="G41" s="29"/>
-      <c r="H41" s="27"/>
+      <c r="B41" s="25"/>
+      <c r="C41" s="26"/>
+      <c r="D41" s="27"/>
+      <c r="E41" s="27"/>
+      <c r="F41" s="31"/>
+      <c r="G41" s="31"/>
+      <c r="H41" s="29"/>
       <c r="I41" s="13"/>
       <c r="J41" s="13"/>
       <c r="K41" s="13"/>
@@ -1885,13 +1904,13 @@
     </row>
     <row r="42" customFormat="false" ht="24.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="13"/>
-      <c r="B42" s="23"/>
-      <c r="C42" s="24"/>
-      <c r="D42" s="25"/>
-      <c r="E42" s="25"/>
-      <c r="F42" s="29"/>
-      <c r="G42" s="29"/>
-      <c r="H42" s="27"/>
+      <c r="B42" s="25"/>
+      <c r="C42" s="26"/>
+      <c r="D42" s="27"/>
+      <c r="E42" s="27"/>
+      <c r="F42" s="31"/>
+      <c r="G42" s="31"/>
+      <c r="H42" s="29"/>
       <c r="I42" s="13"/>
       <c r="J42" s="13"/>
       <c r="K42" s="13"/>
@@ -1909,13 +1928,13 @@
     </row>
     <row r="43" customFormat="false" ht="24.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="13"/>
-      <c r="B43" s="23"/>
-      <c r="C43" s="24"/>
-      <c r="D43" s="25"/>
-      <c r="E43" s="25"/>
-      <c r="F43" s="29"/>
-      <c r="G43" s="29"/>
-      <c r="H43" s="27"/>
+      <c r="B43" s="25"/>
+      <c r="C43" s="26"/>
+      <c r="D43" s="27"/>
+      <c r="E43" s="27"/>
+      <c r="F43" s="31"/>
+      <c r="G43" s="31"/>
+      <c r="H43" s="29"/>
       <c r="I43" s="13"/>
       <c r="J43" s="13"/>
       <c r="K43" s="13"/>
@@ -1933,13 +1952,13 @@
     </row>
     <row r="44" customFormat="false" ht="24.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="13"/>
-      <c r="B44" s="23"/>
-      <c r="C44" s="24"/>
-      <c r="D44" s="25"/>
-      <c r="E44" s="25"/>
-      <c r="F44" s="29"/>
-      <c r="G44" s="29"/>
-      <c r="H44" s="27"/>
+      <c r="B44" s="25"/>
+      <c r="C44" s="26"/>
+      <c r="D44" s="27"/>
+      <c r="E44" s="27"/>
+      <c r="F44" s="31"/>
+      <c r="G44" s="31"/>
+      <c r="H44" s="29"/>
       <c r="I44" s="13"/>
       <c r="J44" s="13"/>
       <c r="K44" s="13"/>
@@ -1957,13 +1976,13 @@
     </row>
     <row r="45" customFormat="false" ht="24.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="13"/>
-      <c r="B45" s="23"/>
-      <c r="C45" s="24"/>
-      <c r="D45" s="25"/>
-      <c r="E45" s="25"/>
-      <c r="F45" s="29"/>
-      <c r="G45" s="29"/>
-      <c r="H45" s="27"/>
+      <c r="B45" s="25"/>
+      <c r="C45" s="26"/>
+      <c r="D45" s="27"/>
+      <c r="E45" s="27"/>
+      <c r="F45" s="31"/>
+      <c r="G45" s="31"/>
+      <c r="H45" s="29"/>
       <c r="I45" s="13"/>
       <c r="J45" s="13"/>
       <c r="K45" s="13"/>
@@ -1981,13 +2000,13 @@
     </row>
     <row r="46" customFormat="false" ht="24.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="13"/>
-      <c r="B46" s="23"/>
-      <c r="C46" s="24"/>
-      <c r="D46" s="25"/>
-      <c r="E46" s="25"/>
-      <c r="F46" s="29"/>
-      <c r="G46" s="29"/>
-      <c r="H46" s="27"/>
+      <c r="B46" s="25"/>
+      <c r="C46" s="26"/>
+      <c r="D46" s="27"/>
+      <c r="E46" s="27"/>
+      <c r="F46" s="31"/>
+      <c r="G46" s="31"/>
+      <c r="H46" s="29"/>
       <c r="I46" s="13"/>
       <c r="J46" s="13"/>
       <c r="K46" s="13"/>
@@ -2005,13 +2024,13 @@
     </row>
     <row r="47" customFormat="false" ht="24.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="13"/>
-      <c r="B47" s="23"/>
-      <c r="C47" s="24"/>
-      <c r="D47" s="25"/>
-      <c r="E47" s="25"/>
-      <c r="F47" s="29"/>
-      <c r="G47" s="29"/>
-      <c r="H47" s="27"/>
+      <c r="B47" s="25"/>
+      <c r="C47" s="26"/>
+      <c r="D47" s="27"/>
+      <c r="E47" s="27"/>
+      <c r="F47" s="31"/>
+      <c r="G47" s="31"/>
+      <c r="H47" s="29"/>
       <c r="I47" s="13"/>
       <c r="J47" s="13"/>
       <c r="K47" s="13"/>
@@ -2029,13 +2048,13 @@
     </row>
     <row r="48" customFormat="false" ht="24.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="13"/>
-      <c r="B48" s="23"/>
-      <c r="C48" s="24"/>
-      <c r="D48" s="25"/>
-      <c r="E48" s="25"/>
-      <c r="F48" s="29"/>
-      <c r="G48" s="29"/>
-      <c r="H48" s="27"/>
+      <c r="B48" s="25"/>
+      <c r="C48" s="26"/>
+      <c r="D48" s="27"/>
+      <c r="E48" s="27"/>
+      <c r="F48" s="31"/>
+      <c r="G48" s="31"/>
+      <c r="H48" s="29"/>
       <c r="I48" s="13"/>
       <c r="J48" s="13"/>
       <c r="K48" s="13"/>
@@ -2053,13 +2072,13 @@
     </row>
     <row r="49" customFormat="false" ht="24.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="13"/>
-      <c r="B49" s="23"/>
-      <c r="C49" s="24"/>
-      <c r="D49" s="25"/>
-      <c r="E49" s="25"/>
-      <c r="F49" s="29"/>
-      <c r="G49" s="29"/>
-      <c r="H49" s="27"/>
+      <c r="B49" s="25"/>
+      <c r="C49" s="26"/>
+      <c r="D49" s="27"/>
+      <c r="E49" s="27"/>
+      <c r="F49" s="31"/>
+      <c r="G49" s="31"/>
+      <c r="H49" s="29"/>
       <c r="I49" s="13"/>
       <c r="J49" s="13"/>
       <c r="K49" s="13"/>
@@ -2077,13 +2096,13 @@
     </row>
     <row r="50" customFormat="false" ht="24.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="13"/>
-      <c r="B50" s="23"/>
-      <c r="C50" s="24"/>
-      <c r="D50" s="25"/>
-      <c r="E50" s="25"/>
-      <c r="F50" s="29"/>
-      <c r="G50" s="29"/>
-      <c r="H50" s="27"/>
+      <c r="B50" s="25"/>
+      <c r="C50" s="26"/>
+      <c r="D50" s="27"/>
+      <c r="E50" s="27"/>
+      <c r="F50" s="31"/>
+      <c r="G50" s="31"/>
+      <c r="H50" s="29"/>
       <c r="I50" s="13"/>
       <c r="J50" s="13"/>
       <c r="K50" s="13"/>
@@ -2101,13 +2120,13 @@
     </row>
     <row r="51" customFormat="false" ht="24.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="13"/>
-      <c r="B51" s="23"/>
-      <c r="C51" s="24"/>
-      <c r="D51" s="25"/>
-      <c r="E51" s="25"/>
-      <c r="F51" s="29"/>
-      <c r="G51" s="29"/>
-      <c r="H51" s="27"/>
+      <c r="B51" s="25"/>
+      <c r="C51" s="26"/>
+      <c r="D51" s="27"/>
+      <c r="E51" s="27"/>
+      <c r="F51" s="31"/>
+      <c r="G51" s="31"/>
+      <c r="H51" s="29"/>
       <c r="I51" s="13"/>
       <c r="J51" s="13"/>
       <c r="K51" s="13"/>
@@ -2125,13 +2144,13 @@
     </row>
     <row r="52" customFormat="false" ht="24.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="13"/>
-      <c r="B52" s="23"/>
-      <c r="C52" s="24"/>
-      <c r="D52" s="25"/>
-      <c r="E52" s="25"/>
-      <c r="F52" s="29"/>
-      <c r="G52" s="29"/>
-      <c r="H52" s="27"/>
+      <c r="B52" s="25"/>
+      <c r="C52" s="26"/>
+      <c r="D52" s="27"/>
+      <c r="E52" s="27"/>
+      <c r="F52" s="31"/>
+      <c r="G52" s="31"/>
+      <c r="H52" s="29"/>
       <c r="I52" s="13"/>
       <c r="J52" s="13"/>
       <c r="K52" s="13"/>
@@ -2149,13 +2168,13 @@
     </row>
     <row r="53" customFormat="false" ht="24.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="13"/>
-      <c r="B53" s="23"/>
-      <c r="C53" s="24"/>
-      <c r="D53" s="25"/>
-      <c r="E53" s="25"/>
-      <c r="F53" s="29"/>
-      <c r="G53" s="29"/>
-      <c r="H53" s="27"/>
+      <c r="B53" s="25"/>
+      <c r="C53" s="26"/>
+      <c r="D53" s="27"/>
+      <c r="E53" s="27"/>
+      <c r="F53" s="31"/>
+      <c r="G53" s="31"/>
+      <c r="H53" s="29"/>
       <c r="I53" s="13"/>
       <c r="J53" s="13"/>
       <c r="K53" s="13"/>
@@ -2173,13 +2192,13 @@
     </row>
     <row r="54" customFormat="false" ht="24.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="13"/>
-      <c r="B54" s="23"/>
-      <c r="C54" s="24"/>
-      <c r="D54" s="25"/>
-      <c r="E54" s="25"/>
-      <c r="F54" s="29"/>
-      <c r="G54" s="29"/>
-      <c r="H54" s="27"/>
+      <c r="B54" s="25"/>
+      <c r="C54" s="26"/>
+      <c r="D54" s="27"/>
+      <c r="E54" s="27"/>
+      <c r="F54" s="31"/>
+      <c r="G54" s="31"/>
+      <c r="H54" s="29"/>
       <c r="I54" s="13"/>
       <c r="J54" s="13"/>
       <c r="K54" s="13"/>
@@ -2197,13 +2216,13 @@
     </row>
     <row r="55" customFormat="false" ht="24.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="13"/>
-      <c r="B55" s="23"/>
-      <c r="C55" s="24"/>
-      <c r="D55" s="25"/>
-      <c r="E55" s="25"/>
-      <c r="F55" s="29"/>
-      <c r="G55" s="29"/>
-      <c r="H55" s="27"/>
+      <c r="B55" s="25"/>
+      <c r="C55" s="26"/>
+      <c r="D55" s="27"/>
+      <c r="E55" s="27"/>
+      <c r="F55" s="31"/>
+      <c r="G55" s="31"/>
+      <c r="H55" s="29"/>
       <c r="I55" s="13"/>
       <c r="J55" s="13"/>
       <c r="K55" s="13"/>
@@ -2221,13 +2240,13 @@
     </row>
     <row r="56" customFormat="false" ht="24.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="13"/>
-      <c r="B56" s="23"/>
-      <c r="C56" s="24"/>
-      <c r="D56" s="25"/>
-      <c r="E56" s="25"/>
-      <c r="F56" s="29"/>
-      <c r="G56" s="29"/>
-      <c r="H56" s="27"/>
+      <c r="B56" s="25"/>
+      <c r="C56" s="26"/>
+      <c r="D56" s="27"/>
+      <c r="E56" s="27"/>
+      <c r="F56" s="31"/>
+      <c r="G56" s="31"/>
+      <c r="H56" s="29"/>
       <c r="I56" s="13"/>
       <c r="J56" s="13"/>
       <c r="K56" s="13"/>
@@ -2245,13 +2264,13 @@
     </row>
     <row r="57" customFormat="false" ht="24.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="13"/>
-      <c r="B57" s="23"/>
-      <c r="C57" s="24"/>
-      <c r="D57" s="25"/>
-      <c r="E57" s="25"/>
-      <c r="F57" s="29"/>
-      <c r="G57" s="29"/>
-      <c r="H57" s="27"/>
+      <c r="B57" s="25"/>
+      <c r="C57" s="26"/>
+      <c r="D57" s="27"/>
+      <c r="E57" s="27"/>
+      <c r="F57" s="31"/>
+      <c r="G57" s="31"/>
+      <c r="H57" s="29"/>
       <c r="I57" s="13"/>
       <c r="J57" s="13"/>
       <c r="K57" s="13"/>
@@ -2269,13 +2288,13 @@
     </row>
     <row r="58" customFormat="false" ht="24.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="13"/>
-      <c r="B58" s="23"/>
-      <c r="C58" s="24"/>
-      <c r="D58" s="25"/>
-      <c r="E58" s="25"/>
-      <c r="F58" s="29"/>
-      <c r="G58" s="29"/>
-      <c r="H58" s="27"/>
+      <c r="B58" s="25"/>
+      <c r="C58" s="26"/>
+      <c r="D58" s="27"/>
+      <c r="E58" s="27"/>
+      <c r="F58" s="31"/>
+      <c r="G58" s="31"/>
+      <c r="H58" s="29"/>
       <c r="I58" s="13"/>
       <c r="J58" s="13"/>
       <c r="K58" s="13"/>
@@ -2293,13 +2312,13 @@
     </row>
     <row r="59" customFormat="false" ht="24.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="13"/>
-      <c r="B59" s="23"/>
-      <c r="C59" s="24"/>
-      <c r="D59" s="25"/>
-      <c r="E59" s="25"/>
-      <c r="F59" s="29"/>
-      <c r="G59" s="29"/>
-      <c r="H59" s="27"/>
+      <c r="B59" s="25"/>
+      <c r="C59" s="26"/>
+      <c r="D59" s="27"/>
+      <c r="E59" s="27"/>
+      <c r="F59" s="31"/>
+      <c r="G59" s="31"/>
+      <c r="H59" s="29"/>
       <c r="I59" s="13"/>
       <c r="J59" s="13"/>
       <c r="K59" s="13"/>
@@ -2317,13 +2336,13 @@
     </row>
     <row r="60" customFormat="false" ht="24.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="13"/>
-      <c r="B60" s="23"/>
-      <c r="C60" s="24"/>
-      <c r="D60" s="25"/>
-      <c r="E60" s="25"/>
-      <c r="F60" s="29"/>
-      <c r="G60" s="29"/>
-      <c r="H60" s="27"/>
+      <c r="B60" s="25"/>
+      <c r="C60" s="26"/>
+      <c r="D60" s="27"/>
+      <c r="E60" s="27"/>
+      <c r="F60" s="31"/>
+      <c r="G60" s="31"/>
+      <c r="H60" s="29"/>
       <c r="I60" s="13"/>
       <c r="J60" s="13"/>
       <c r="K60" s="13"/>
@@ -2341,13 +2360,13 @@
     </row>
     <row r="61" customFormat="false" ht="24.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="13"/>
-      <c r="B61" s="23"/>
-      <c r="C61" s="24"/>
-      <c r="D61" s="25"/>
-      <c r="E61" s="25"/>
-      <c r="F61" s="29"/>
-      <c r="G61" s="29"/>
-      <c r="H61" s="27"/>
+      <c r="B61" s="25"/>
+      <c r="C61" s="26"/>
+      <c r="D61" s="27"/>
+      <c r="E61" s="27"/>
+      <c r="F61" s="31"/>
+      <c r="G61" s="31"/>
+      <c r="H61" s="29"/>
       <c r="I61" s="13"/>
       <c r="J61" s="13"/>
       <c r="K61" s="13"/>
@@ -2365,13 +2384,13 @@
     </row>
     <row r="62" customFormat="false" ht="24.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="13"/>
-      <c r="B62" s="23"/>
-      <c r="C62" s="24"/>
-      <c r="D62" s="25"/>
-      <c r="E62" s="25"/>
-      <c r="F62" s="29"/>
-      <c r="G62" s="29"/>
-      <c r="H62" s="27"/>
+      <c r="B62" s="25"/>
+      <c r="C62" s="26"/>
+      <c r="D62" s="27"/>
+      <c r="E62" s="27"/>
+      <c r="F62" s="31"/>
+      <c r="G62" s="31"/>
+      <c r="H62" s="29"/>
       <c r="I62" s="13"/>
       <c r="J62" s="13"/>
       <c r="K62" s="13"/>
@@ -2389,13 +2408,13 @@
     </row>
     <row r="63" customFormat="false" ht="24.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="13"/>
-      <c r="B63" s="23"/>
-      <c r="C63" s="24"/>
-      <c r="D63" s="25"/>
-      <c r="E63" s="25"/>
-      <c r="F63" s="29"/>
-      <c r="G63" s="29"/>
-      <c r="H63" s="27"/>
+      <c r="B63" s="25"/>
+      <c r="C63" s="26"/>
+      <c r="D63" s="27"/>
+      <c r="E63" s="27"/>
+      <c r="F63" s="31"/>
+      <c r="G63" s="31"/>
+      <c r="H63" s="29"/>
       <c r="I63" s="13"/>
       <c r="J63" s="13"/>
       <c r="K63" s="13"/>
@@ -2413,13 +2432,13 @@
     </row>
     <row r="64" customFormat="false" ht="24.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="13"/>
-      <c r="B64" s="23"/>
-      <c r="C64" s="30"/>
-      <c r="D64" s="25"/>
-      <c r="E64" s="25"/>
-      <c r="F64" s="29"/>
-      <c r="G64" s="29"/>
-      <c r="H64" s="27"/>
+      <c r="B64" s="25"/>
+      <c r="C64" s="32"/>
+      <c r="D64" s="27"/>
+      <c r="E64" s="27"/>
+      <c r="F64" s="31"/>
+      <c r="G64" s="31"/>
+      <c r="H64" s="29"/>
       <c r="I64" s="13"/>
       <c r="J64" s="13"/>
       <c r="K64" s="13"/>
@@ -2437,13 +2456,13 @@
     </row>
     <row r="65" customFormat="false" ht="24.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="13"/>
-      <c r="B65" s="23"/>
-      <c r="C65" s="24"/>
-      <c r="D65" s="25"/>
-      <c r="E65" s="25"/>
-      <c r="F65" s="29"/>
-      <c r="G65" s="29"/>
-      <c r="H65" s="27"/>
+      <c r="B65" s="25"/>
+      <c r="C65" s="26"/>
+      <c r="D65" s="27"/>
+      <c r="E65" s="27"/>
+      <c r="F65" s="31"/>
+      <c r="G65" s="31"/>
+      <c r="H65" s="29"/>
       <c r="I65" s="13"/>
       <c r="J65" s="13"/>
       <c r="K65" s="13"/>
@@ -2461,13 +2480,13 @@
     </row>
     <row r="66" customFormat="false" ht="24.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="13"/>
-      <c r="B66" s="23"/>
-      <c r="C66" s="24"/>
-      <c r="D66" s="25"/>
-      <c r="E66" s="25"/>
-      <c r="F66" s="29"/>
-      <c r="G66" s="29"/>
-      <c r="H66" s="27"/>
+      <c r="B66" s="25"/>
+      <c r="C66" s="26"/>
+      <c r="D66" s="27"/>
+      <c r="E66" s="27"/>
+      <c r="F66" s="31"/>
+      <c r="G66" s="31"/>
+      <c r="H66" s="29"/>
       <c r="I66" s="13"/>
       <c r="J66" s="13"/>
       <c r="K66" s="13"/>
@@ -2485,13 +2504,13 @@
     </row>
     <row r="67" customFormat="false" ht="24.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="13"/>
-      <c r="B67" s="23"/>
-      <c r="C67" s="24"/>
-      <c r="D67" s="25"/>
-      <c r="E67" s="25"/>
-      <c r="F67" s="29"/>
-      <c r="G67" s="29"/>
-      <c r="H67" s="27"/>
+      <c r="B67" s="25"/>
+      <c r="C67" s="26"/>
+      <c r="D67" s="27"/>
+      <c r="E67" s="27"/>
+      <c r="F67" s="31"/>
+      <c r="G67" s="31"/>
+      <c r="H67" s="29"/>
       <c r="I67" s="13"/>
       <c r="J67" s="13"/>
       <c r="K67" s="13"/>
@@ -2509,13 +2528,13 @@
     </row>
     <row r="68" customFormat="false" ht="24.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="13"/>
-      <c r="B68" s="23"/>
-      <c r="C68" s="24"/>
-      <c r="D68" s="25"/>
-      <c r="E68" s="25"/>
-      <c r="F68" s="29"/>
-      <c r="G68" s="29"/>
-      <c r="H68" s="27"/>
+      <c r="B68" s="25"/>
+      <c r="C68" s="26"/>
+      <c r="D68" s="27"/>
+      <c r="E68" s="27"/>
+      <c r="F68" s="31"/>
+      <c r="G68" s="31"/>
+      <c r="H68" s="29"/>
       <c r="I68" s="13"/>
       <c r="J68" s="13"/>
       <c r="K68" s="13"/>
@@ -2533,13 +2552,13 @@
     </row>
     <row r="69" customFormat="false" ht="24.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="13"/>
-      <c r="B69" s="23"/>
-      <c r="C69" s="24"/>
-      <c r="D69" s="25"/>
-      <c r="E69" s="25"/>
-      <c r="F69" s="29"/>
-      <c r="G69" s="29"/>
-      <c r="H69" s="27"/>
+      <c r="B69" s="25"/>
+      <c r="C69" s="26"/>
+      <c r="D69" s="27"/>
+      <c r="E69" s="27"/>
+      <c r="F69" s="31"/>
+      <c r="G69" s="31"/>
+      <c r="H69" s="29"/>
       <c r="I69" s="13"/>
       <c r="J69" s="13"/>
       <c r="K69" s="13"/>
@@ -2557,13 +2576,13 @@
     </row>
     <row r="70" customFormat="false" ht="24.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="13"/>
-      <c r="B70" s="23"/>
-      <c r="C70" s="24"/>
-      <c r="D70" s="25"/>
-      <c r="E70" s="25"/>
-      <c r="F70" s="29"/>
-      <c r="G70" s="29"/>
-      <c r="H70" s="27"/>
+      <c r="B70" s="25"/>
+      <c r="C70" s="26"/>
+      <c r="D70" s="27"/>
+      <c r="E70" s="27"/>
+      <c r="F70" s="31"/>
+      <c r="G70" s="31"/>
+      <c r="H70" s="29"/>
       <c r="I70" s="13"/>
       <c r="J70" s="13"/>
       <c r="K70" s="13"/>
@@ -2581,13 +2600,13 @@
     </row>
     <row r="71" customFormat="false" ht="24.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="13"/>
-      <c r="B71" s="23"/>
-      <c r="C71" s="24"/>
-      <c r="D71" s="25"/>
-      <c r="E71" s="25"/>
-      <c r="F71" s="29"/>
-      <c r="G71" s="29"/>
-      <c r="H71" s="27"/>
+      <c r="B71" s="25"/>
+      <c r="C71" s="26"/>
+      <c r="D71" s="27"/>
+      <c r="E71" s="27"/>
+      <c r="F71" s="31"/>
+      <c r="G71" s="31"/>
+      <c r="H71" s="29"/>
       <c r="I71" s="13"/>
       <c r="J71" s="13"/>
       <c r="K71" s="13"/>
@@ -2605,13 +2624,13 @@
     </row>
     <row r="72" customFormat="false" ht="24.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="13"/>
-      <c r="B72" s="23"/>
-      <c r="C72" s="24"/>
-      <c r="D72" s="25"/>
-      <c r="E72" s="25"/>
-      <c r="F72" s="29"/>
-      <c r="G72" s="29"/>
-      <c r="H72" s="27"/>
+      <c r="B72" s="25"/>
+      <c r="C72" s="26"/>
+      <c r="D72" s="27"/>
+      <c r="E72" s="27"/>
+      <c r="F72" s="31"/>
+      <c r="G72" s="31"/>
+      <c r="H72" s="29"/>
       <c r="I72" s="13"/>
       <c r="J72" s="13"/>
       <c r="K72" s="13"/>
@@ -2629,13 +2648,13 @@
     </row>
     <row r="73" customFormat="false" ht="24.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="13"/>
-      <c r="B73" s="23"/>
-      <c r="C73" s="24"/>
-      <c r="D73" s="25"/>
-      <c r="E73" s="25"/>
-      <c r="F73" s="29"/>
-      <c r="G73" s="29"/>
-      <c r="H73" s="27"/>
+      <c r="B73" s="25"/>
+      <c r="C73" s="26"/>
+      <c r="D73" s="27"/>
+      <c r="E73" s="27"/>
+      <c r="F73" s="31"/>
+      <c r="G73" s="31"/>
+      <c r="H73" s="29"/>
       <c r="I73" s="13"/>
       <c r="J73" s="13"/>
       <c r="K73" s="13"/>
@@ -2653,13 +2672,13 @@
     </row>
     <row r="74" customFormat="false" ht="24.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="13"/>
-      <c r="B74" s="23"/>
-      <c r="C74" s="24"/>
-      <c r="D74" s="25"/>
-      <c r="E74" s="25"/>
-      <c r="F74" s="29"/>
-      <c r="G74" s="29"/>
-      <c r="H74" s="27"/>
+      <c r="B74" s="25"/>
+      <c r="C74" s="26"/>
+      <c r="D74" s="27"/>
+      <c r="E74" s="27"/>
+      <c r="F74" s="31"/>
+      <c r="G74" s="31"/>
+      <c r="H74" s="29"/>
       <c r="I74" s="13"/>
       <c r="J74" s="13"/>
       <c r="K74" s="13"/>
@@ -2677,13 +2696,13 @@
     </row>
     <row r="75" customFormat="false" ht="24.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="13"/>
-      <c r="B75" s="23"/>
-      <c r="C75" s="24"/>
-      <c r="D75" s="25"/>
-      <c r="E75" s="25"/>
-      <c r="F75" s="29"/>
-      <c r="G75" s="29"/>
-      <c r="H75" s="27"/>
+      <c r="B75" s="25"/>
+      <c r="C75" s="26"/>
+      <c r="D75" s="27"/>
+      <c r="E75" s="27"/>
+      <c r="F75" s="31"/>
+      <c r="G75" s="31"/>
+      <c r="H75" s="29"/>
       <c r="I75" s="13"/>
       <c r="J75" s="13"/>
       <c r="K75" s="13"/>
@@ -2701,13 +2720,13 @@
     </row>
     <row r="76" customFormat="false" ht="24.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="13"/>
-      <c r="B76" s="31"/>
-      <c r="C76" s="24"/>
-      <c r="D76" s="25"/>
-      <c r="E76" s="25"/>
-      <c r="F76" s="29"/>
-      <c r="G76" s="29"/>
-      <c r="H76" s="27"/>
+      <c r="B76" s="33"/>
+      <c r="C76" s="26"/>
+      <c r="D76" s="27"/>
+      <c r="E76" s="27"/>
+      <c r="F76" s="31"/>
+      <c r="G76" s="31"/>
+      <c r="H76" s="29"/>
       <c r="I76" s="13"/>
       <c r="J76" s="13"/>
       <c r="K76" s="13"/>
@@ -2935,7 +2954,7 @@
       <formula1>AND(ISNUMBER(LEFT(I1,FIND(":",I1&amp;":")-1)+0),ISNUMBER(MID(I1,FIND(":",I1&amp;":")+1,LEN(I1))+0),ISNUMBER(FIND(":",I1)))</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="greaterThanOrEqual" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="F5:G36" type="whole">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="greaterThanOrEqual" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="F5:G13 K5:K12 F14:G36" type="whole">
       <formula1>0</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -2966,77 +2985,77 @@
   <dimension ref="A1:B11"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="95.07"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14.09"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="95.07"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="14.09"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="24.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="32" t="s">
-        <v>24</v>
-      </c>
-      <c r="B1" s="32" t="s">
+      <c r="A1" s="34" t="s">
         <v>25</v>
       </c>
+      <c r="B1" s="34" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="33" t="s">
-        <v>26</v>
-      </c>
-      <c r="B2" s="33" t="n">
+      <c r="A2" s="35" t="s">
+        <v>27</v>
+      </c>
+      <c r="B2" s="35" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="B3" s="33" t="n">
+      <c r="A3" s="35" t="s">
+        <v>28</v>
+      </c>
+      <c r="B3" s="35" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="33" t="s">
-        <v>28</v>
-      </c>
-      <c r="B4" s="33" t="n">
+      <c r="A4" s="35" t="s">
+        <v>29</v>
+      </c>
+      <c r="B4" s="35" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="34"/>
-      <c r="B5" s="34"/>
+      <c r="A5" s="36"/>
+      <c r="B5" s="36"/>
     </row>
     <row r="6" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="34"/>
-      <c r="B6" s="34"/>
+      <c r="A6" s="36"/>
+      <c r="B6" s="36"/>
     </row>
     <row r="7" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="34"/>
-      <c r="B7" s="34"/>
+      <c r="A7" s="36"/>
+      <c r="B7" s="36"/>
     </row>
     <row r="8" customFormat="false" ht="24.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="35" t="s">
-        <v>29</v>
-      </c>
-      <c r="B8" s="34"/>
+      <c r="A8" s="37" t="s">
+        <v>30</v>
+      </c>
+      <c r="B8" s="36"/>
     </row>
     <row r="9" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="34" t="s">
-        <v>30</v>
-      </c>
-      <c r="B9" s="34"/>
+      <c r="A9" s="36" t="s">
+        <v>31</v>
+      </c>
+      <c r="B9" s="36"/>
     </row>
     <row r="10" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="34" t="s">
-        <v>31</v>
-      </c>
-      <c r="B10" s="34"/>
+      <c r="A10" s="36" t="s">
+        <v>32</v>
+      </c>
+      <c r="B10" s="36"/>
     </row>
     <row r="11" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="34" t="s">
-        <v>32</v>
-      </c>
-      <c r="B11" s="34"/>
+      <c r="A11" s="36" t="s">
+        <v>33</v>
+      </c>
+      <c r="B11" s="36"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>